<commit_message>
Export quotidien 2026-06-15 [mois_courant]
</commit_message>
<xml_diff>
--- a/_data_mois.xlsx
+++ b/_data_mois.xlsx
@@ -487,10 +487,10 @@
         <v>2026</v>
       </c>
       <c r="C2" t="n">
-        <v>35066.73</v>
+        <v>35469.48</v>
       </c>
       <c r="D2" t="n">
-        <v>9868.1</v>
+        <v>10270.85</v>
       </c>
       <c r="E2" t="n">
         <v>25198.63</v>
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>10387.78</v>
+        <v>10790.53</v>
       </c>
     </row>
     <row r="5">
@@ -667,7 +667,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>4565.9</v>
+        <v>4968.65</v>
       </c>
     </row>
     <row r="7">
@@ -912,7 +912,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Paramétrages</t>
+          <t>Clôture</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -924,7 +924,7 @@
         <v>895</v>
       </c>
       <c r="L3" t="n">
-        <v>492.25</v>
+        <v>895</v>
       </c>
     </row>
     <row r="4">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>[DEPARTEMENT D'ILLE ET VILAINE (CD 35)] - Montée de version Littéralis - 1 journée d'assistance fonctionnelle à distance</t>
+          <t>[CD 35)] - Montée de version Littéralis - 1 journée d'assistance fonctionnelle à distance</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>[CONSEIL DEPARTEMENTAL DE LA SAVOIE (CD 73)] - Purge arrêtés temporaires</t>
+          <t>[CD 73)] - Purge arrêtés temporaires</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2053,19 +2053,19 @@
         <v>2026</v>
       </c>
       <c r="C2" t="n">
-        <v>150.25</v>
+        <v>154</v>
       </c>
       <c r="D2" t="n">
-        <v>21.75</v>
+        <v>23.25</v>
       </c>
       <c r="E2" t="n">
-        <v>66.5</v>
+        <v>71</v>
       </c>
       <c r="F2" t="n">
         <v>11.5</v>
       </c>
       <c r="G2" t="n">
-        <v>35.5</v>
+        <v>37</v>
       </c>
       <c r="H2" t="n">
         <v>5.5</v>

</xml_diff>